<commit_message>
Initial commit: Parts 1-3 complete
</commit_message>
<xml_diff>
--- a/pubmed_aptamer_thrombin.xlsx
+++ b/pubmed_aptamer_thrombin.xlsx
@@ -453,220 +453,220 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>42242804</t>
+          <t>39321910</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Programmable Fc-encoded DNA tile-cube capture enables a thrombin-activated ratiometric ECL/SERS biosensor via a PAM-engineered toehold switch and CRISPR/Cas12a cleavage.</t>
+          <t>Aptamer biosensors for thrombin.</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Accurate thrombin detection is important for coagulation-related assessment, but reliable quantification at ultralow levels remains challenging because matrix interference, electrode-to-electrode variation, and single-channel signal drift can compromise analytical accuracy. Herein, we developed a thrombin-responsive ratiometric electrochemiluminescence/surface-enhanced Raman scattering (ECL/SERS) biosensor integrating Fc-encoded DNA tiles, a DNA-cube capture scaffold, and a PAM-engineered toehold-switch-regulated CRISPR/Cas12a module on a Ti An intentionally cleavable linker probe (LP) serves as the bridge for retaining Fc-rich DNA tiles near the electrode. Without thrombin, intact LP enables tile capture, causing ECL quenching and strong Fc SERS output. With thrombin, split-aptamer proximity assembly activates the toehold switch and Cas12a/crRNA, leading to LP cleavage, Fc-tile depletion, ECL recovery, and SERS attenuation. The anti-correlated signals were integrated as Q = I This work establishes a programmable capture-release strategy that converts thrombin recognition into CRISPR/Cas12a-mediated LP cleavage and deterministic interfacial reconfiguration, providing a sensitive, internally referenced, and extensible platform for protein biosensing.</t>
+          <t>Thrombin, a key factor in the coagulation cascade, is a valuable biomarker of great importance for the prognosis, diagnosis, and monitoring of various diseases, including cancer and heart disease. Due to the increasing attention to the development of point-of-care testing (POCT) options, various types of biosensors have been invented to enhance the accuracy and speed of detection of important biomarkers such as thrombin. Implementation of aptamers in biosensors (aptasensors) improves the target recognition capacity due to the high-affinity binding nature of aptamers. Herein, this review presents recent studies of aptasensors for thrombin detection based on different detection mechanisms encompassing optical biosensors, surface-enhanced Raman spectroscopy (SERS), electrochemical detection, piezoelectric detection, and lateral flow assay.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>42237925</t>
+          <t>38502201</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Assembly of Protein-DNA Framework Nanostructures: Structurally Defining Protein-DNA Interfaces With Aptamer.</t>
+          <t>Sandwich-type aptamer-based biosensors for thrombin detection.</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>DNA and proteins have been extensively explored for self-assembly of nanostructures. Each has its own advantages and limitations. By integrating them together, protein-DNA frameworks (PDFs) could potentially combine their advantages while overcoming the limitations associated with each component; thus, providing a huge diversity in terms of structures, functionalities, assembly versatilities, and responsiveness. Though each has been demonstrated to self-assemble into large structures, it remains a great challenge to engineer well-structured protein-DNA interfaces for PDF assembly. Herein, we report a robust and versatile approach to this problem. Specific and high-affinity protein-aptamer binding can nicely interface protein and DNA with structural control. A series of bivalent thrombin aptamers were designed to co-assemble with thrombin into a range of PDFs including discrete triangles and 3D prisms, linear and circular oligomers, 1D chains/ladders, and 2D arrays. The versatility of such a strategy was further demonstrated by the self-assembly of Plasmodium falciparum lactate dehydrogenase (PfLDH)-containing PDFs. In this work, AlphaFold 3, a universal modeling program, dramatically facilitates structural modeling and helps the designs. We believe that such a rational PDF design will find wide applications as multimodal biomaterials integrating the diverse functionalities of proteins and the ease of assembly programmability of DNA.</t>
+          <t>Thrombin, a proteolytic enzyme, plays an essential role in catalyzing many blood clotting reactions. Thrombin can act as a marker for some blood-related diseases, such as leukemia, thrombosis, Alzheimer's disease and liver disease. Therefore, its diagnosis is of great importance in the fields of biological and medical research. Biosensors containing sandwich-type structures have attracted much consideration owing to their superior features such as reproducible and stable responses with easy improvement in the sensitivity of detection. Sandwich-type platforms can be designed using a pair of receptors that are able to bind to diverse locations of the same target. Herein, we investigate recent advances in the progress and applications of thrombin aptasensors containing a sandwich-type structure, in which two thrombin-binding aptamers (TBAs) identify different parts of the thrombin molecule, leading to the formation of a sandwich structure and ultimately signal detection. We also discuss the pros and cons of these approaches and outline the most logical approach in each section.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2024</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>42224769</t>
+          <t>19377993</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>SELEX-derived potassium aptamers for robust detection in a physiological sodium background.</t>
+          <t>Aptamers and biosensors.</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Potassium (K</t>
+          <t>The immobilization procedure to a biosensor surface has a major influence on the measurement results. To characterize the immobilization onto various biolayers, the interaction of DNA anti-thrombin aptamer with the protein thrombin was used as a model system. The aptamer was immobilized to a two-dimensional alkanethiol SAM via carboxylamide bonds and to a three-dimensional dextran matrix via streptavidin-biotin interaction. The calculated K (D) values of about 260 and 267 nM, respectively, were comparable, while the amount of bound analyte varied by a factor of 2, depending on the accessibility of the immobilized aptamer. Differences in the specificity were shown by use of the similar protein elastase.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2009</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>42194045</t>
+          <t>32777331</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Effects of Loop Nucleobase Substitution on G-Quadruplex Thermal Stability in Aqueous Glycine Betaine, Proline, TMAO, and Urea Solutions.</t>
+          <t>G-quadruplex-based aptamers targeting human thrombin: Discovery, chemical modifications and antithrombotic effects.</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>G-quadruplexes are guanine-rich DNA or RNA structures comprising two or more stacked guanine tetrads (G-quartet) with nucleobases in the loops linking the G-quartets. The thermal stability of the thrombin-binding aptamer G2 d(G</t>
+          <t>First studies on thrombin-inhibiting DNA aptamers were reported in 1992, and since then a large number of anticoagulant aptamers has been discovered. TBA - also named HD1, a 15-mer G-quadruplex (G4)-forming oligonucleotide - is the best characterized thrombin binding aptamer, able to specifically recognize the protein exosite I, thus inhibiting the conversion of soluble fibrinogen into insoluble fibrin strands. Unmodified nucleic acid-based aptamers, in general, and TBA in particular, exhibit limited pharmacokinetic properties and are rapidly degraded in vivo by nucleases. In order to improve the biological performance of aptamers, a widely investigated strategy is the introduction of chemical modifications in their backbone at the level of the nucleobases, sugar moieties or phosphodiester linkages. Besides TBA, also other thrombin binding aptamers, able to adopt a well-defined G4 structure, e.g. mixed duplex/quadruplex sequences, as well as homo- and hetero-bivalent constructs, have been identified and optimized. Considering the growing need of new efficient anticoagulant agents associated with the strong therapeutic potential of these thrombin inhibitors, the research on thrombin binding aptamers is still a very hot and intriguing field. Herein, we comprehensively described the state-of-the-art knowledge on the DNA-based aptamers targeting thrombin, especially focusing on the optimized analogues obtained by chemically modifying the oligonucleotide backbone, and their biological performances in therapeutic applications.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2021</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>42149311</t>
+          <t>30015643</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Protein-protein interaction disruption as a next-generation antithrombotic strategy.</t>
+          <t>Emerging applications of aptamers for anticoagulation and hemostasis.</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Thrombosis is built, not merely catalyzed. Across arterial and venous disease, thrombus formation depends on a succession of protein-protein interactions (PPIs) that coordinate platelet capture and activation, thromboinflammatory amplification, and assembly of membrane-bound coagulation complexes. Although active-site inhibitors and receptor antagonists have transformed antithrombotic therapy, clinical benefit is often constrained by bleeding because many targets are indispensable for everyday hemostasis when inhibited systemically. This review advances a "thrombus assembly" framework that reframes drug discovery around disrupting interfaces that organize pathologic clot growth in a context-dependent manner shaped by shear, surfaces, local cofactors, and transient complex formation. We highlight translational proof that interface blockade works in humans, focusing on VWF A1-GPIbα inhibition and GPVI-directed strategies as exemplars of lesion- and shear-dependent antiplatelet therapy. We then survey platelet adhesion and activation PPIs (VWF-GPIb, collagen-GPVI, and αIIbβ3-ligand interactions), thromboinflammatory interfaces (including P-selectin-PSGL-1 and CLEC-2-podoplanin), and opportunities to target coagulation complex assembly and thrombin exosites without directly inhibiting catalytic active sites. A modality-focused section links interface class to therapeutic format-antibodies/nanobodies, aptamers with antidotes, peptides and macrocycles, and small-molecule PPI inhibitors-and summarizes trade-offs in reversibility, half-life, manufacturability, and immunogenicity. Finally, we discuss assays that preserve interface biology (whole-blood flow systems, microfluidics, thrombin generation, and clot mechanics) and propose clinical positioning and trial endpoints for context-gated mechanisms. By targeting the contacts that assemble and stabilize thrombi, PPI disruption offers a pragmatic route toward more selective, potentially bleeding-sparing antithrombotic therapy and a roadmap for next-generation pipeline development.</t>
+          <t>Since the selection of the first thrombin-binding aptamer in 1992, the use of nucleic acid aptamers to target specific coagulation factors has emerged as a valuable approach for generating novel anticoagulant and procoagulant therapeutics. Herein, we highlight the most recent discoveries involving application of aptamers for those purposes. Learning from the successes and pitfalls of the FIXa-targeting aptamer pegnivacogin in preclinical and clinical studies, the latest efforts to develop antidote-controllable anticoagulation strategies for cardiopulmonary bypass that avoid unfractionated heparin involve potentiation of the exosite-binding factor X (FX)a aptamer 11F7t by combination with either a small molecule FXa catalytic site inhibitor or a thrombin aptamer. Recent work has also focused on identifying aptamer inhibitors of contact pathway factors such as FXIa and kallikrein, which may prove to be well tolerated and effective antithrombotic agents in certain clinical settings. Finally, new approaches to develop procoagulant aptamers to control bleeding associated with hemophilia and other coagulopathies involve targeting activated protein C and tissue plasminogen activator. Overall, these recent findings exemplify the versatility of aptamers to modulate a variety of procoagulant and anticoagulant factors, along with their capacity to be used complementarily with other aptamers or drugs for wide-ranging applications.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2018</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>42146644</t>
+          <t>25483931</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Aptamer-based DNA nanoswitches for multiplexed protein detection.</t>
+          <t>Anomeric DNA quadruplexes.</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Simple, modular platforms for detecting biologically relevant proteins are critical for applications in clinical diagnostics, healthcare, and research. Here, we have combined aptamer-based protein recognition with our conformationally-responsive DNA nanoswitches to enable simple, sensitive and specific protein detection. We demonstrate dual detection of two clinically relevant blood proteins, thrombin and VEGF as initial proof of concept.</t>
+          <t>Thrombin-binding aptamer (TBA) is a 15-nt DNA oligomer that efficiently inhibits thrombin. It has been shown that TBA folds into an anti-parallel unimolecular G-quadruplex. Its three-dimensional chair-like structure consists of two G-tetrads connected by TT and TGT loops. TBA undergoes fast degradation by nucleases in vivo. To improve the nuclease resistance of TBA, a number of modified analogs have been proposed. Here, we describe anomeric modifications of TBA. Non-natural α anomers were used to replace selected nucleotides in the loops and core. Significant stabilization of the quadruplex was observed for the anomeric modification of TT loops at T4 and T13. Replacement of the core guanines either prevents quadruplex assembly or induces rearrangement in G-tetrads. It was found that the anticoagulant properties of chimeric aptamers could be retained only with intact TT loops. On the contrary, modification of the TGT loop was shown to substantially increase nuclease resistance of the chimeric aptamer without a notable disturbance of its anticoagulant activity.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2014</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>42101160</t>
+          <t>36948709</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Brush-on-Brush Architecture Enables Durable and Reversible Aptamer Therapeutics With Minimal PEG Associated Immunogenicity.</t>
+          <t>Protein labeling and crosslinking by covalent aptamers.</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>We present a "Brush-on-Brush" (BOB) nanocarrier as a next-generation alternative to PEGylation for nucleic acid aptamer therapeutics. This architecture, comprising aptamers and dense brush-shaped oligo(ethylene glycol) (b-OEG) side chains co-grafted onto a peptide backbone, was validated using the thrombin-binding HD1 aptamer. BOB-HD1 exhibited exceptional nuclease resistance, retaining &gt;40% integrity after 2 h of S1 nuclease exposure (versus complete degradation of free aptamer within 3 min), while fully preserving G-quadruplex folding, thrombin-binding activity, and antidote-mediated reversibility. In mice, BOB-HD1 achieved a 7.5-fold increase in systemic exposure and sustained anticoagulation for 4 h, compared to &lt;20 min for unmodified or linearly PEGylated aptamer. Critically, unlike linear PEG conjugates that induced anti-PEG antibodies and accelerated blood clearance upon repeated dosing, BOB-HD1 induced no detectable anti PEG IgM or IgG responses under the tested conditions and maintained full efficacy upon repeated administration. This dense brush architecture thus addresses key stability, clearance, and PEG associated immunogenicity barriers that have impeded aptamer clinical translation, offering a versatile and controllable platform for durable aptamer therapeutics while minimizing detectable anti PEG antibody responses under the tested conditions.</t>
+          <t>In this chapter, a new approach to the selective modification of native proteins is discussed, using electrophilic covalent aptamers. These biochemical tools are generated through the site-specific incorporation of a label-transferring or crosslinking electrophile into a DNA aptamer. Covalent aptamers provide the ability to transfer a variety of functional handles to a protein of interest or to irreversibly crosslink to the target. Methods for the aptamer-mediated labeling and crosslinking of thrombin are described. Thrombin labeling is fast and selective, in both simple buffer and in human plasma and outcompetes nuclease-mediated degradation. This approach provides facile, sensitive detection of labeled protein by western blot, SDS-PAGE, and mass spectrometry.</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2023</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>42068939</t>
+          <t>37326345</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Electrochemical biosensor for ultrasensitive thrombin detection based on aptamer-modulated transcriptional inhibition of cell-free synthetic biology.</t>
+          <t>Nucleic acid aptamer-based biosensors and their application in thrombin analysis.</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>In this study, a novel strategy integrating aptamer-gated cell-free synthetic biology with electrochemical analysis has been developed for thrombin detection (using thrombin as a model target). A DNA template embedded with a target-specific aptamer is designed as a "molecular switch". Target binding induces a conformational change in the aptamer, creating steric hindrance for T7 RNA polymerase and thereby inhibiting transcription of the RNA reporter strand. The transcribed RNA can hybridize with methylene blue (MB)-labeled DNA probes immobilized on the electrode surface, causing electroactive species to move away from the electrode surface and resulting in a relatively low electrochemical signal. Conversely, a reduced amount of transcribed RNA leads to an increased electrochemical signal. Under optimized conditions, the biosensor exhibits a linear range of 0.06 nM - 6 μM and a limit of detection (LOD) of 0.032 nM (S/N = 3). The sensor demonstrates excellent specificity against interfering proteins. Spike-recovery tests in 20-fold diluted human serum yield recoveries of 95.35% - 105.20% with RSD values of 2.32% - 4.90%, confirming its anti-interference ability in complex biological matrices. This methodological innovation realizes sensitive and specific detection of thrombin and provides a generalizable strategy for cell-free electrochemical analysis of protein targets. By replacing the aptamer sequence, the platform can be extended to diverse proteins, opening new avenues for the application of cell-free synthetic biology in biosensing and clinical diagnostics.</t>
+          <t>Thrombin is a multifunctional serine protease that plays an important role in coagulation and anticoagulation processes. Aptamers have been widely applied in biosensors due to their high specificity, low cost and good biocompatibility. This review summarizes recent advances in thrombin quantification using aptamer-based biosensors. The primary focus is optical sensors and electrochemical sensors, along with their applications in thrombin analysis and disease diagnosis.</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2023</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>42063839</t>
+          <t>35013452</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Paranemic Cohesion of DNA under Isothermal Conditions.</t>
+          <t>Structure-guided development of Pb</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Recent progress in DNA nanotechnology has shown the isothermal assembly of several DNA nanostructures. Isothermal assembly allows DNA nanostructure construction in a variety of ions while simplifying DNA nanotechnology by avoiding the need for thermal cyclers and expands utility by enabling attachment of guest biomolecules on DNA nanostructures at ambient or physiological temperatures. The paranemic crossover (PX) DNA motif has been used in the construction of DNA nanostructures, paranemic cohesion has been used to connect DNA structures as an alternate to sticky end cohesion, and PX DNA has also been implied to have a biological role in homology recognition. In that context, here we demonstrate the successful isothermal assembly of the PX DNA motif in magnesium (Mg</t>
+          <t>Owing to its great threat to human health and environment, Pb</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2022</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>42062222</t>
+          <t>22376117</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Switchable DNA-Scaffolded Multivalent Aptamer through Stimuli-Responsive Plug-and-Play Modules for Protein Regulation.</t>
+          <t>G-quadruplex DNA aptamers and their ligands: structure, function and application.</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Multivalent molecular interactions enhance binding affinity and enable functional regulation in biological systems, inspiring the development of multivalent materials for biosensing and biomedical applications. The capacity to reversibly switch between low-valency and multivalency as needed is key to regulating their function. However, current design strategies face challenges in enabling such switching within the same system through a response to multiple stimuli. Here, as a proof of concept, we demonstrate a switchable multivalent system for regulating thrombin activity. This system is based on thrombin aptamer-decorated DNA tile assembly and introduces stimuli-responsive plug-and-play modules that serve as dynamic, reversible, and orthogonal switches responding to the corresponding stimuli, including UV light, APE1, and RNase H. We construct three-layer switching cascades activated by one-, two-, or three stimuli to regulate thrombin activity. Building upon this programmable multivalent aptamer system, we further translate switchable modules into spatiotemporal control logic to construct a tristate circuit. We hope that the switchable DNA scaffold-based multivalent regulatory approach can provide a versatile modular platform with potential applications in precision medicine, biosensing, and biomaterials.</t>
+          <t>Highly specific and tight-binding nucleic acid aptamers have been selected against a variety of molecular targets for over 20 years. A significant proportion of these oligonucleotides display G-quadruplex structures, particularly for DNA aptamers, that enable molecular recognition of their ligands. G-quadruplex structures couple a common scaffold to varying loop motifs that act in target recognition. Here, we review DNA G-quadruplex aptamers and their ligands from a structural and functional perspective. We compare the diversity of DNA G-quadruplex aptamers selected against multiple ligand targets, and consider structure with a particular focus on dissecting the thrombin binding aptamer - thrombin interaction. Therapeutic and analytical applications of DNA G-quadruplex aptamers are also discussed. Understanding DNA G-quadruplex aptamers carries implications not only for therapeutics and diagnostics, but also in the natural biochemistry of guanine-rich nucleic acids.</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2012</t>
         </is>
       </c>
     </row>

</xml_diff>